<commit_message>
Completed telemetry mapping sheet with field details
</commit_message>
<xml_diff>
--- a/telemetry_mapping_sheet.xlsx
+++ b/telemetry_mapping_sheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\madhu\Desktop\Infotact-project1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5237C101-FC8F-4F69-8075-32BF723FAD48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB0D7E9B-4774-4BE4-A697-F7260CED86D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{DA5FBD98-07F2-40D4-85CF-A14B82AF09F0}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{DA5FBD98-07F2-40D4-85CF-A14B82AF09F0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="33">
   <si>
     <t>Source Field</t>
   </si>
@@ -49,6 +49,90 @@
   </si>
   <si>
     <t>Data Type</t>
+  </si>
+  <si>
+    <t>Timestamp</t>
+  </si>
+  <si>
+    <t>TIMESTAMP</t>
+  </si>
+  <si>
+    <t>Direct</t>
+  </si>
+  <si>
+    <t>Timestamp when telemetry data was generated</t>
+  </si>
+  <si>
+    <t>Container_ID</t>
+  </si>
+  <si>
+    <t>VARCHAR</t>
+  </si>
+  <si>
+    <t>Unique identifier of the shipping container</t>
+  </si>
+  <si>
+    <t>Cargo_Type</t>
+  </si>
+  <si>
+    <t>Type of cargo being transported</t>
+  </si>
+  <si>
+    <t>Origin</t>
+  </si>
+  <si>
+    <t>Shipment origin location</t>
+  </si>
+  <si>
+    <t>Destination</t>
+  </si>
+  <si>
+    <t>Shipment destination location</t>
+  </si>
+  <si>
+    <t>Temperature_C</t>
+  </si>
+  <si>
+    <t>FLOAT</t>
+  </si>
+  <si>
+    <t>Temperature inside the container (°C)</t>
+  </si>
+  <si>
+    <t>Humidity_Percent</t>
+  </si>
+  <si>
+    <t>Humidity level inside the container (%)</t>
+  </si>
+  <si>
+    <t>Vibration_Level</t>
+  </si>
+  <si>
+    <t>Vibration sensor reading during transport</t>
+  </si>
+  <si>
+    <t>Distance_Remaining_km</t>
+  </si>
+  <si>
+    <t>Remaining distance to the destination (km)</t>
+  </si>
+  <si>
+    <t>Spoilage_Risk</t>
+  </si>
+  <si>
+    <t>Estimated spoilage risk level</t>
+  </si>
+  <si>
+    <t>Recommended_Action</t>
+  </si>
+  <si>
+    <t>Suggested action based on telemetry data</t>
+  </si>
+  <si>
+    <t>Alert_Status</t>
+  </si>
+  <si>
+    <t>Current alert status of the shipment</t>
   </si>
 </sst>
 </file>
@@ -92,9 +176,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -409,7 +496,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA39AB37-67B1-4105-883E-18EA0D6CC8FB}">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.44140625" customWidth="1"/>
@@ -436,6 +523,210 @@
         <v>3</v>
       </c>
     </row>
+    <row r="2" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Improved telemetry mapping sheet
</commit_message>
<xml_diff>
--- a/telemetry_mapping_sheet.xlsx
+++ b/telemetry_mapping_sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\madhu\Desktop\Infotact-project1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB0D7E9B-4774-4BE4-A697-F7260CED86D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28513601-9A63-47BB-969F-03286E48B45F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{DA5FBD98-07F2-40D4-85CF-A14B82AF09F0}"/>
   </bookViews>
@@ -176,11 +176,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -496,14 +504,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA39AB37-67B1-4105-883E-18EA0D6CC8FB}">
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.44140625" customWidth="1"/>
-    <col min="2" max="2" width="13.33203125" customWidth="1"/>
-    <col min="3" max="3" width="9.88671875" customWidth="1"/>
-    <col min="4" max="4" width="12.44140625" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="1" max="1" width="20.109375" customWidth="1"/>
+    <col min="2" max="2" width="21" customWidth="1"/>
+    <col min="3" max="3" width="15.5546875" customWidth="1"/>
+    <col min="4" max="4" width="19.77734375" customWidth="1"/>
+    <col min="5" max="5" width="43.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
@@ -523,209 +531,212 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="4" t="s">
         <v>7</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="4" t="s">
         <v>7</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>12</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="4" t="s">
         <v>7</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>14</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="4" t="s">
         <v>7</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="4" t="s">
         <v>7</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>18</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="4" t="s">
         <v>7</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>21</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="4" t="s">
         <v>7</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>23</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="4" t="s">
         <v>7</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>25</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="4" t="s">
         <v>7</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>27</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="D11" s="4" t="s">
         <v>7</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>29</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="D12" s="4" t="s">
         <v>7</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>31</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C13" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="D13" s="4" t="s">
         <v>7</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>32</v>
       </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>